<commit_message>
Read Smart Store links from xlsx instead of a manual map
xlsx now has a 5th column (사이트링크) with one representative URL per
product line filled in by hand. build-products.py reads it directly -
one non-empty URL anywhere in a line's rows becomes that line's url,
since color/size variants share one Smart Store page. Invalid entries
(non-http values, e.g. a stray typo) are dropped with a warning instead
of silently kept. URL_MAP is now just a fallback for lines that don't
exist in the xlsx (e.g. flower-class).

19 of 25 lines have links so far; 6 are still empty and get listed on
every run. Prices are unchanged in this update - only urls were added.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/테차상품가격리스트.xlsx
+++ b/docs/테차상품가격리스트.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\사업장\26년테차\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764C0D55-41EA-4462-B1D8-B961A6B80652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45F81D1E-1101-4125-9956-5256BB93F19D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4BF26195-36F7-4BB5-9460-51DA0CA0C59D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="190">
   <si>
     <t>상품</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -1087,6 +1087,68 @@
   <si>
     <t>추천용도</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>사이트링크</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/6202622460</t>
+  </si>
+  <si>
+    <t>ㅍ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/10663209995</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/6205690862</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/8528473340</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/6563272914</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/12333689454</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/10968901786</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/7090535704</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/6506821191</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/6622301544</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/6957075209</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/8424617454</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/9333901539</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/9614048648</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/12236511010</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/13346419874</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/13355757045</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/13337020734</t>
   </si>
 </sst>
 </file>
@@ -1363,7 +1425,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
@@ -1692,16 +1754,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B63D9B1D-9853-4DE5-AF47-C6E10EB25A9C}">
-  <dimension ref="A1:D148"/>
+  <dimension ref="A1:E148"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="59.5" customWidth="1"/>
     <col min="2" max="2" width="14.75" style="1" customWidth="1"/>
     <col min="3" max="3" width="31.25" customWidth="1"/>
     <col min="4" max="4" width="59.875" customWidth="1"/>
+    <col min="5" max="5" width="55.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.25">
+    <row r="1" spans="1:5" ht="20.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1714,8 +1777,11 @@
       <c r="D1" s="19" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="10" t="s">
         <v>2</v>
       </c>
@@ -1725,8 +1791,11 @@
       <c r="C2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -1737,7 +1806,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
@@ -1748,7 +1817,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
@@ -1759,7 +1828,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="A6" s="10" t="s">
         <v>6</v>
       </c>
@@ -1770,7 +1839,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:5">
       <c r="A7" s="10" t="s">
         <v>7</v>
       </c>
@@ -1781,7 +1850,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:5">
       <c r="A8" s="10" t="s">
         <v>8</v>
       </c>
@@ -1792,7 +1861,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:5">
       <c r="A9" s="10" t="s">
         <v>9</v>
       </c>
@@ -1803,7 +1872,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:5">
       <c r="A10" s="10" t="s">
         <v>10</v>
       </c>
@@ -1814,7 +1883,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:5">
       <c r="A11" s="10" t="s">
         <v>11</v>
       </c>
@@ -1825,7 +1894,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:5">
       <c r="A12" s="10" t="s">
         <v>12</v>
       </c>
@@ -1836,7 +1905,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:5">
       <c r="A13" s="10" t="s">
         <v>13</v>
       </c>
@@ -1847,7 +1916,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:5">
       <c r="A14" s="10" t="s">
         <v>14</v>
       </c>
@@ -1858,7 +1927,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:5">
       <c r="A15" s="10" t="s">
         <v>15</v>
       </c>
@@ -1869,7 +1938,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:5">
       <c r="A16" s="6" t="s">
         <v>16</v>
       </c>
@@ -1879,8 +1948,11 @@
       <c r="C16" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="E16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" s="6" t="s">
         <v>17</v>
       </c>
@@ -1891,7 +1963,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:5">
       <c r="A18" s="6" t="s">
         <v>18</v>
       </c>
@@ -1902,7 +1974,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:5">
       <c r="A19" s="6" t="s">
         <v>19</v>
       </c>
@@ -1913,7 +1985,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:5">
       <c r="A20" s="6" t="s">
         <v>20</v>
       </c>
@@ -1924,7 +1996,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:5">
       <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
@@ -1935,7 +2007,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:5">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -1946,7 +2018,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:5">
       <c r="A23" s="6" t="s">
         <v>23</v>
       </c>
@@ -1957,7 +2029,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:5">
       <c r="A24" s="6" t="s">
         <v>24</v>
       </c>
@@ -1968,7 +2040,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:5">
       <c r="A25" s="6" t="s">
         <v>25</v>
       </c>
@@ -1979,7 +2051,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:5">
       <c r="A26" s="6" t="s">
         <v>26</v>
       </c>
@@ -1990,7 +2062,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:5">
       <c r="A27" s="6" t="s">
         <v>27</v>
       </c>
@@ -2001,7 +2073,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:5">
       <c r="A28" s="6" t="s">
         <v>28</v>
       </c>
@@ -2012,7 +2084,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:5">
       <c r="A29" s="5" t="s">
         <v>111</v>
       </c>
@@ -2022,8 +2094,11 @@
       <c r="C29" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
+      <c r="E29" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" s="5" t="s">
         <v>112</v>
       </c>
@@ -2034,7 +2109,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:5">
       <c r="A31" s="5" t="s">
         <v>113</v>
       </c>
@@ -2045,7 +2120,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:5">
       <c r="A32" s="5" t="s">
         <v>114</v>
       </c>
@@ -2056,7 +2131,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:5">
       <c r="A33" s="6" t="s">
         <v>29</v>
       </c>
@@ -2066,8 +2141,11 @@
       <c r="C33" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="E33" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34" s="6" t="s">
         <v>30</v>
       </c>
@@ -2078,7 +2156,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:5">
       <c r="A35" s="6" t="s">
         <v>31</v>
       </c>
@@ -2089,7 +2167,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:5">
       <c r="A36" s="6" t="s">
         <v>32</v>
       </c>
@@ -2100,7 +2178,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:5">
       <c r="A37" s="6" t="s">
         <v>33</v>
       </c>
@@ -2111,7 +2189,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:5">
       <c r="A38" s="6" t="s">
         <v>34</v>
       </c>
@@ -2122,7 +2200,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:5">
       <c r="A39" s="6" t="s">
         <v>35</v>
       </c>
@@ -2133,7 +2211,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:5">
       <c r="A40" s="6" t="s">
         <v>36</v>
       </c>
@@ -2144,7 +2222,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:5">
       <c r="A41" s="5" t="s">
         <v>136</v>
       </c>
@@ -2155,7 +2233,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:5">
       <c r="A42" s="5" t="s">
         <v>137</v>
       </c>
@@ -2165,8 +2243,11 @@
       <c r="C42" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="43" spans="1:3">
+      <c r="E42" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
       <c r="A43" s="5" t="s">
         <v>138</v>
       </c>
@@ -2177,7 +2258,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:5">
       <c r="A44" s="5" t="s">
         <v>139</v>
       </c>
@@ -2188,7 +2269,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:5">
       <c r="A45" s="5" t="s">
         <v>140</v>
       </c>
@@ -2199,7 +2280,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:5">
       <c r="A46" s="5" t="s">
         <v>141</v>
       </c>
@@ -2210,7 +2291,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:5">
       <c r="A47" s="5" t="s">
         <v>142</v>
       </c>
@@ -2221,7 +2302,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:5">
       <c r="A48" s="5" t="s">
         <v>143</v>
       </c>
@@ -2232,7 +2313,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:5">
       <c r="A49" s="10" t="s">
         <v>37</v>
       </c>
@@ -2242,8 +2323,11 @@
       <c r="C49" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
+      <c r="E49" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
       <c r="A50" s="10" t="s">
         <v>38</v>
       </c>
@@ -2254,7 +2338,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:5">
       <c r="A51" s="10" t="s">
         <v>39</v>
       </c>
@@ -2265,7 +2349,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:5">
       <c r="A52" s="10" t="s">
         <v>41</v>
       </c>
@@ -2276,7 +2360,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:5">
       <c r="A53" s="10" t="s">
         <v>42</v>
       </c>
@@ -2287,7 +2371,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:5">
       <c r="A54" s="10" t="s">
         <v>40</v>
       </c>
@@ -2298,7 +2382,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:5">
       <c r="A55" s="10" t="s">
         <v>44</v>
       </c>
@@ -2309,7 +2393,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:5">
       <c r="A56" s="10" t="s">
         <v>45</v>
       </c>
@@ -2320,7 +2404,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:5">
       <c r="A57" s="10" t="s">
         <v>43</v>
       </c>
@@ -2331,7 +2415,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:5">
       <c r="A58" s="10" t="s">
         <v>46</v>
       </c>
@@ -2342,7 +2426,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:5">
       <c r="A59" s="10" t="s">
         <v>47</v>
       </c>
@@ -2353,7 +2437,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:5">
       <c r="A60" s="10" t="s">
         <v>48</v>
       </c>
@@ -2364,7 +2448,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:5">
       <c r="A61" s="8" t="s">
         <v>58</v>
       </c>
@@ -2374,8 +2458,11 @@
       <c r="C61" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
+      <c r="E61" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
       <c r="A62" s="8" t="s">
         <v>59</v>
       </c>
@@ -2386,7 +2473,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:5">
       <c r="A63" s="8" t="s">
         <v>60</v>
       </c>
@@ -2397,7 +2484,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:5">
       <c r="A64" s="8" t="s">
         <v>61</v>
       </c>
@@ -2408,7 +2495,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:5">
       <c r="A65" s="8" t="s">
         <v>62</v>
       </c>
@@ -2419,7 +2506,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:5">
       <c r="A66" s="8" t="s">
         <v>63</v>
       </c>
@@ -2430,7 +2517,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:5">
       <c r="A67" s="8" t="s">
         <v>64</v>
       </c>
@@ -2441,7 +2528,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:5">
       <c r="A68" s="8" t="s">
         <v>65</v>
       </c>
@@ -2452,7 +2539,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:5">
       <c r="A69" s="8" t="s">
         <v>66</v>
       </c>
@@ -2463,7 +2550,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:5">
       <c r="A70" s="8" t="s">
         <v>67</v>
       </c>
@@ -2474,7 +2561,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:5">
       <c r="A71" s="8" t="s">
         <v>68</v>
       </c>
@@ -2485,7 +2572,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:5">
       <c r="A72" s="8" t="s">
         <v>69</v>
       </c>
@@ -2496,7 +2583,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:5">
       <c r="A73" s="12" t="s">
         <v>49</v>
       </c>
@@ -2506,8 +2593,11 @@
       <c r="C73" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="74" spans="1:3">
+      <c r="E73" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
       <c r="A74" s="12" t="s">
         <v>50</v>
       </c>
@@ -2518,7 +2608,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:5">
       <c r="A75" s="12" t="s">
         <v>51</v>
       </c>
@@ -2529,7 +2619,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:5">
       <c r="A76" s="6" t="s">
         <v>119</v>
       </c>
@@ -2539,8 +2629,11 @@
       <c r="C76" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="77" spans="1:3">
+      <c r="E76" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
       <c r="A77" s="6" t="s">
         <v>118</v>
       </c>
@@ -2551,7 +2644,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:5">
       <c r="A78" s="6" t="s">
         <v>120</v>
       </c>
@@ -2562,7 +2655,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:5">
       <c r="A79" s="6" t="s">
         <v>121</v>
       </c>
@@ -2573,7 +2666,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:5">
       <c r="A80" s="4" t="s">
         <v>52</v>
       </c>
@@ -2583,8 +2676,11 @@
       <c r="C80" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="81" spans="1:3">
+      <c r="E80" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
       <c r="A81" s="5" t="s">
         <v>53</v>
       </c>
@@ -2595,7 +2691,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:5">
       <c r="A82" s="5" t="s">
         <v>54</v>
       </c>
@@ -2606,7 +2702,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:5">
       <c r="A83" s="5" t="s">
         <v>55</v>
       </c>
@@ -2617,7 +2713,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:5">
       <c r="A84" s="5" t="s">
         <v>56</v>
       </c>
@@ -2628,7 +2724,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:5">
       <c r="A85" s="5" t="s">
         <v>57</v>
       </c>
@@ -2639,7 +2735,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:5">
       <c r="A86" s="7" t="s">
         <v>70</v>
       </c>
@@ -2649,8 +2745,11 @@
       <c r="C86" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="87" spans="1:3">
+      <c r="E86" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
       <c r="A87" s="8" t="s">
         <v>71</v>
       </c>
@@ -2661,7 +2760,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:5">
       <c r="A88" s="8" t="s">
         <v>72</v>
       </c>
@@ -2672,7 +2771,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:5">
       <c r="A89" s="8" t="s">
         <v>73</v>
       </c>
@@ -2683,7 +2782,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:5">
       <c r="A90" s="8" t="s">
         <v>74</v>
       </c>
@@ -2694,7 +2793,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:5">
       <c r="A91" s="8" t="s">
         <v>75</v>
       </c>
@@ -2705,7 +2804,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:5">
       <c r="A92" s="8" t="s">
         <v>76</v>
       </c>
@@ -2716,7 +2815,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:5">
       <c r="A93" s="8" t="s">
         <v>77</v>
       </c>
@@ -2727,7 +2826,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:5">
       <c r="A94" s="9" t="s">
         <v>78</v>
       </c>
@@ -2737,8 +2836,11 @@
       <c r="C94" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="95" spans="1:3">
+      <c r="E94" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
       <c r="A95" s="10" t="s">
         <v>79</v>
       </c>
@@ -2749,7 +2851,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:5">
       <c r="A96" s="10" t="s">
         <v>80</v>
       </c>
@@ -2760,7 +2862,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:5">
       <c r="A97" s="10" t="s">
         <v>81</v>
       </c>
@@ -2771,7 +2873,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:5">
       <c r="A98" s="10" t="s">
         <v>82</v>
       </c>
@@ -2782,7 +2884,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:5">
       <c r="A99" s="10" t="s">
         <v>83</v>
       </c>
@@ -2793,7 +2895,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:5">
       <c r="A100" s="10" t="s">
         <v>84</v>
       </c>
@@ -2804,7 +2906,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:5">
       <c r="A101" s="10" t="s">
         <v>85</v>
       </c>
@@ -2815,7 +2917,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:5">
       <c r="A102" s="11" t="s">
         <v>86</v>
       </c>
@@ -2825,8 +2927,11 @@
       <c r="C102" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="103" spans="1:3">
+      <c r="E102" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5">
       <c r="A103" s="12" t="s">
         <v>87</v>
       </c>
@@ -2837,7 +2942,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:5">
       <c r="A104" s="12" t="s">
         <v>88</v>
       </c>
@@ -2848,7 +2953,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:5">
       <c r="A105" s="12" t="s">
         <v>89</v>
       </c>
@@ -2859,7 +2964,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:5">
       <c r="A106" s="12" t="s">
         <v>90</v>
       </c>
@@ -2870,7 +2975,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:5">
       <c r="A107" s="12" t="s">
         <v>91</v>
       </c>
@@ -2881,7 +2986,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:5">
       <c r="A108" s="12" t="s">
         <v>92</v>
       </c>
@@ -2892,7 +2997,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:5">
       <c r="A109" s="12" t="s">
         <v>93</v>
       </c>
@@ -2903,7 +3008,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:5">
       <c r="A110" s="13" t="s">
         <v>94</v>
       </c>
@@ -2913,8 +3018,11 @@
       <c r="C110" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="111" spans="1:3">
+      <c r="E110" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5">
       <c r="A111" s="6" t="s">
         <v>95</v>
       </c>
@@ -2925,7 +3033,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:5">
       <c r="A112" s="6" t="s">
         <v>96</v>
       </c>
@@ -2936,7 +3044,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:5">
       <c r="A113" s="6" t="s">
         <v>97</v>
       </c>
@@ -2947,7 +3055,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:5">
       <c r="A114" s="5" t="s">
         <v>101</v>
       </c>
@@ -2957,8 +3065,11 @@
       <c r="C114" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="115" spans="1:3">
+      <c r="E114" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5">
       <c r="A115" s="5" t="s">
         <v>102</v>
       </c>
@@ -2969,7 +3080,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:5">
       <c r="A116" s="5" t="s">
         <v>100</v>
       </c>
@@ -2980,7 +3091,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:5">
       <c r="A117" s="4" t="s">
         <v>98</v>
       </c>
@@ -2991,7 +3102,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:5">
       <c r="A118" s="5" t="s">
         <v>99</v>
       </c>
@@ -3002,7 +3113,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:5">
       <c r="A119" s="7" t="s">
         <v>103</v>
       </c>
@@ -3012,8 +3123,11 @@
       <c r="C119" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="120" spans="1:3">
+      <c r="E119" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5">
       <c r="A120" s="8" t="s">
         <v>104</v>
       </c>
@@ -3024,7 +3138,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:5">
       <c r="A121" s="8" t="s">
         <v>105</v>
       </c>
@@ -3035,7 +3149,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:5">
       <c r="A122" s="9" t="s">
         <v>106</v>
       </c>
@@ -3046,7 +3160,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:5">
       <c r="A123" s="10" t="s">
         <v>107</v>
       </c>
@@ -3056,8 +3170,11 @@
       <c r="C123" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="124" spans="1:3">
+      <c r="E123" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5">
       <c r="A124" s="10" t="s">
         <v>108</v>
       </c>
@@ -3068,7 +3185,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:5">
       <c r="A125" s="10" t="s">
         <v>109</v>
       </c>
@@ -3079,7 +3196,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:5">
       <c r="A126" s="10" t="s">
         <v>110</v>
       </c>
@@ -3090,7 +3207,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:5">
       <c r="A127" s="11" t="s">
         <v>115</v>
       </c>
@@ -3100,8 +3217,11 @@
       <c r="C127" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="128" spans="1:3">
+      <c r="E127" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5">
       <c r="A128" s="12" t="s">
         <v>116</v>
       </c>
@@ -3112,7 +3232,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="17.25" thickBot="1">
+    <row r="129" spans="1:5" ht="17.25" thickBot="1">
       <c r="A129" s="12" t="s">
         <v>117</v>
       </c>
@@ -3123,7 +3243,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="17.25" thickBot="1">
+    <row r="130" spans="1:5" ht="17.25" thickBot="1">
       <c r="A130" s="17" t="s">
         <v>145</v>
       </c>
@@ -3133,8 +3253,11 @@
       <c r="C130" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" ht="17.25" thickBot="1">
+      <c r="E130" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" ht="17.25" thickBot="1">
       <c r="A131" s="17" t="s">
         <v>146</v>
       </c>
@@ -3145,7 +3268,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="17.25" thickBot="1">
+    <row r="132" spans="1:5" ht="17.25" thickBot="1">
       <c r="A132" s="17" t="s">
         <v>147</v>
       </c>
@@ -3156,7 +3279,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="17.25" thickBot="1">
+    <row r="133" spans="1:5" ht="17.25" thickBot="1">
       <c r="A133" s="17" t="s">
         <v>148</v>
       </c>
@@ -3167,7 +3290,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="17.25" thickBot="1">
+    <row r="134" spans="1:5" ht="17.25" thickBot="1">
       <c r="A134" s="17" t="s">
         <v>149</v>
       </c>
@@ -3178,7 +3301,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="17.25" thickBot="1">
+    <row r="135" spans="1:5" ht="17.25" thickBot="1">
       <c r="A135" s="17" t="s">
         <v>150</v>
       </c>
@@ -3189,7 +3312,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="17.25" thickBot="1">
+    <row r="136" spans="1:5" ht="17.25" thickBot="1">
       <c r="A136" s="14" t="s">
         <v>122</v>
       </c>
@@ -3199,8 +3322,11 @@
       <c r="C136" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" ht="17.25" thickBot="1">
+      <c r="E136" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" ht="17.25" thickBot="1">
       <c r="A137" s="14" t="s">
         <v>123</v>
       </c>
@@ -3211,7 +3337,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="17.25" thickBot="1">
+    <row r="138" spans="1:5" ht="17.25" thickBot="1">
       <c r="A138" s="14" t="s">
         <v>124</v>
       </c>
@@ -3222,7 +3348,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="17.25" thickBot="1">
+    <row r="139" spans="1:5" ht="17.25" thickBot="1">
       <c r="A139" s="14" t="s">
         <v>125</v>
       </c>
@@ -3233,7 +3359,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="17.25" thickBot="1">
+    <row r="140" spans="1:5" ht="17.25" thickBot="1">
       <c r="A140" s="14" t="s">
         <v>126</v>
       </c>
@@ -3244,7 +3370,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="17.25" thickBot="1">
+    <row r="141" spans="1:5" ht="17.25" thickBot="1">
       <c r="A141" s="14" t="s">
         <v>127</v>
       </c>
@@ -3255,7 +3381,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="17.25" thickBot="1">
+    <row r="142" spans="1:5" ht="17.25" thickBot="1">
       <c r="A142" s="14" t="s">
         <v>128</v>
       </c>
@@ -3266,7 +3392,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="17.25" thickBot="1">
+    <row r="143" spans="1:5" ht="17.25" thickBot="1">
       <c r="A143" s="14" t="s">
         <v>129</v>
       </c>
@@ -3277,7 +3403,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="17.25" thickBot="1">
+    <row r="144" spans="1:5" ht="17.25" thickBot="1">
       <c r="A144" s="14" t="s">
         <v>130</v>
       </c>
@@ -3288,7 +3414,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="17.25" thickBot="1">
+    <row r="145" spans="1:5" ht="17.25" thickBot="1">
       <c r="A145" s="14" t="s">
         <v>131</v>
       </c>
@@ -3299,7 +3425,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="17.25" thickBot="1">
+    <row r="146" spans="1:5" ht="17.25" thickBot="1">
       <c r="A146" s="14" t="s">
         <v>132</v>
       </c>
@@ -3310,7 +3436,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="17.25" thickBot="1">
+    <row r="147" spans="1:5" ht="17.25" thickBot="1">
       <c r="A147" s="14" t="s">
         <v>133</v>
       </c>
@@ -3321,7 +3447,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="148" spans="1:3">
+    <row r="148" spans="1:5">
       <c r="A148" s="15" t="s">
         <v>134</v>
       </c>
@@ -3330,6 +3456,9 @@
       </c>
       <c r="C148" t="s">
         <v>167</v>
+      </c>
+      <c r="E148" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix rose-soap-bouquet link (was a stray typo, now the real URL)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/테차상품가격리스트.xlsx
+++ b/docs/테차상품가격리스트.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45F81D1E-1101-4125-9956-5256BB93F19D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF09C943-3049-4A87-B169-95935D2EEEA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4BF26195-36F7-4BB5-9460-51DA0CA0C59D}"/>
   </bookViews>
@@ -1096,10 +1096,6 @@
     <t>https://smartstore.naver.com/itecha/products/6202622460</t>
   </si>
   <si>
-    <t>ㅍ</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>https://smartstore.naver.com/itecha/products/10663209995</t>
   </si>
   <si>
@@ -1149,6 +1145,9 @@
   </si>
   <si>
     <t>https://smartstore.naver.com/itecha/products/13337020734</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/itecha/products/7563519851</t>
   </si>
 </sst>
 </file>
@@ -1159,7 +1158,7 @@
     <numFmt numFmtId="6" formatCode="&quot;₩&quot;#,##0;[Red]\-&quot;₩&quot;#,##0"/>
     <numFmt numFmtId="176" formatCode="&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1324,6 +1323,12 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1379,7 +1384,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1438,6 +1443,9 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1948,8 +1956,8 @@
       <c r="C16" t="s">
         <v>144</v>
       </c>
-      <c r="E16" t="s">
-        <v>172</v>
+      <c r="E16" s="20" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2095,7 +2103,7 @@
         <v>135</v>
       </c>
       <c r="E29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2142,7 +2150,7 @@
         <v>144</v>
       </c>
       <c r="E33" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2244,7 +2252,7 @@
         <v>144</v>
       </c>
       <c r="E42" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2324,7 +2332,7 @@
         <v>144</v>
       </c>
       <c r="E49" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -2459,7 +2467,7 @@
         <v>151</v>
       </c>
       <c r="E61" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -2594,7 +2602,7 @@
         <v>152</v>
       </c>
       <c r="E73" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -2630,7 +2638,7 @@
         <v>152</v>
       </c>
       <c r="E76" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -2677,7 +2685,7 @@
         <v>154</v>
       </c>
       <c r="E80" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -2746,7 +2754,7 @@
         <v>155</v>
       </c>
       <c r="E86" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -2837,7 +2845,7 @@
         <v>155</v>
       </c>
       <c r="E94" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -2928,7 +2936,7 @@
         <v>155</v>
       </c>
       <c r="E102" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -3019,7 +3027,7 @@
         <v>156</v>
       </c>
       <c r="E110" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -3066,7 +3074,7 @@
         <v>157</v>
       </c>
       <c r="E114" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -3124,7 +3132,7 @@
         <v>158</v>
       </c>
       <c r="E119" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -3171,7 +3179,7 @@
         <v>160</v>
       </c>
       <c r="E123" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -3218,7 +3226,7 @@
         <v>164</v>
       </c>
       <c r="E127" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -3254,7 +3262,7 @@
         <v>165</v>
       </c>
       <c r="E130" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="131" spans="1:5" ht="17.25" thickBot="1">
@@ -3323,7 +3331,7 @@
         <v>166</v>
       </c>
       <c r="E136" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="137" spans="1:5" ht="17.25" thickBot="1">
@@ -3458,7 +3466,7 @@
         <v>167</v>
       </c>
       <c r="E148" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>